<commit_message>
Added new file plus minor code updates
</commit_message>
<xml_diff>
--- a/Data/Rules/Adored Beast Rules Matrix.xlsx
+++ b/Data/Rules/Adored Beast Rules Matrix.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="78">
   <si>
     <t>SKU</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t>HQ_Max</t>
+  </si>
+  <si>
+    <t>Total Max</t>
   </si>
   <si>
     <t>29109</t>
@@ -576,10 +579,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN19"/>
+  <dimension ref="A1:AO19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:40">
+    <row r="1" spans="1:41">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -700,16 +703,19 @@
       <c r="AN1" t="s">
         <v>39</v>
       </c>
+      <c r="AO1" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="2" spans="1:40">
+    <row r="2" spans="1:41">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -822,16 +828,19 @@
       <c r="AN2">
         <v>0</v>
       </c>
+      <c r="AO2">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:40">
+    <row r="3" spans="1:41">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -944,16 +953,19 @@
       <c r="AN3">
         <v>0</v>
       </c>
+      <c r="AO3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:40">
+    <row r="4" spans="1:41">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1066,16 +1078,19 @@
       <c r="AN4">
         <v>0</v>
       </c>
+      <c r="AO4">
+        <v>24</v>
+      </c>
     </row>
-    <row r="5" spans="1:40">
+    <row r="5" spans="1:41">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1188,16 +1203,19 @@
       <c r="AN5">
         <v>0</v>
       </c>
+      <c r="AO5">
+        <v>17</v>
+      </c>
     </row>
-    <row r="6" spans="1:40">
+    <row r="6" spans="1:41">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1310,16 +1328,19 @@
       <c r="AN6">
         <v>0</v>
       </c>
+      <c r="AO6">
+        <v>26</v>
+      </c>
     </row>
-    <row r="7" spans="1:40">
+    <row r="7" spans="1:41">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1432,16 +1453,19 @@
       <c r="AN7">
         <v>0</v>
       </c>
+      <c r="AO7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:40">
+    <row r="8" spans="1:41">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1554,16 +1578,19 @@
       <c r="AN8">
         <v>0</v>
       </c>
+      <c r="AO8">
+        <v>29</v>
+      </c>
     </row>
-    <row r="9" spans="1:40">
+    <row r="9" spans="1:41">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1676,16 +1703,19 @@
       <c r="AN9">
         <v>0</v>
       </c>
+      <c r="AO9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:40">
+    <row r="10" spans="1:41">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1798,16 +1828,19 @@
       <c r="AN10">
         <v>0</v>
       </c>
+      <c r="AO10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:40">
+    <row r="11" spans="1:41">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1920,16 +1953,19 @@
       <c r="AN11">
         <v>0</v>
       </c>
+      <c r="AO11">
+        <v>32</v>
+      </c>
     </row>
-    <row r="12" spans="1:40">
+    <row r="12" spans="1:41">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -2042,16 +2078,19 @@
       <c r="AN12">
         <v>0</v>
       </c>
+      <c r="AO12">
+        <v>30</v>
+      </c>
     </row>
-    <row r="13" spans="1:40">
+    <row r="13" spans="1:41">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -2164,16 +2203,19 @@
       <c r="AN13">
         <v>0</v>
       </c>
+      <c r="AO13">
+        <v>21</v>
+      </c>
     </row>
-    <row r="14" spans="1:40">
+    <row r="14" spans="1:41">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -2286,16 +2328,19 @@
       <c r="AN14">
         <v>0</v>
       </c>
+      <c r="AO14">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:40">
+    <row r="15" spans="1:41">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -2408,382 +2453,394 @@
       <c r="AN15">
         <v>0</v>
       </c>
+      <c r="AO15">
+        <v>21</v>
+      </c>
     </row>
-    <row r="16" spans="1:40">
+    <row r="16" spans="1:41">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>2</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>2</v>
+      </c>
+      <c r="K16" t="b">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>2</v>
+      </c>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="b">
+        <v>1</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <v>1</v>
+      </c>
+      <c r="V16">
+        <v>2</v>
+      </c>
+      <c r="W16" t="b">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>1</v>
+      </c>
+      <c r="Y16">
+        <v>2</v>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16">
+        <v>1</v>
+      </c>
+      <c r="AB16">
+        <v>1</v>
+      </c>
+      <c r="AC16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD16">
+        <v>1</v>
+      </c>
+      <c r="AE16">
+        <v>1</v>
+      </c>
+      <c r="AF16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG16">
+        <v>1</v>
+      </c>
+      <c r="AH16">
+        <v>2</v>
+      </c>
+      <c r="AI16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ16">
+        <v>1</v>
+      </c>
+      <c r="AK16">
+        <v>1</v>
+      </c>
+      <c r="AL16" t="b">
+        <v>1</v>
+      </c>
+      <c r="AM16">
+        <v>0</v>
+      </c>
+      <c r="AN16">
+        <v>0</v>
+      </c>
+      <c r="AO16">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:41">
+      <c r="A17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" t="s">
+        <v>77</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17" t="b">
+        <v>1</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="b">
+        <v>1</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17" t="b">
+        <v>1</v>
+      </c>
+      <c r="U17">
+        <v>0</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17">
+        <v>0</v>
+      </c>
+      <c r="Y17">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA17">
+        <v>0</v>
+      </c>
+      <c r="AB17">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+      <c r="AE17">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG17">
+        <v>0</v>
+      </c>
+      <c r="AH17">
+        <v>0</v>
+      </c>
+      <c r="AI17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AJ17">
+        <v>0</v>
+      </c>
+      <c r="AK17">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AM17">
+        <v>0</v>
+      </c>
+      <c r="AN17">
+        <v>0</v>
+      </c>
+      <c r="AO17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:41">
+      <c r="A18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+      <c r="K18" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>2</v>
+      </c>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18">
+        <v>1</v>
+      </c>
+      <c r="Q18" t="b">
+        <v>1</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18" t="b">
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <v>1</v>
+      </c>
+      <c r="V18">
+        <v>2</v>
+      </c>
+      <c r="W18" t="b">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>1</v>
+      </c>
+      <c r="Y18">
+        <v>1</v>
+      </c>
+      <c r="Z18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA18">
+        <v>1</v>
+      </c>
+      <c r="AB18">
+        <v>1</v>
+      </c>
+      <c r="AC18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD18">
+        <v>1</v>
+      </c>
+      <c r="AE18">
+        <v>1</v>
+      </c>
+      <c r="AF18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG18">
+        <v>1</v>
+      </c>
+      <c r="AH18">
+        <v>2</v>
+      </c>
+      <c r="AI18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ18">
+        <v>1</v>
+      </c>
+      <c r="AK18">
+        <v>1</v>
+      </c>
+      <c r="AL18" t="b">
+        <v>1</v>
+      </c>
+      <c r="AM18">
+        <v>0</v>
+      </c>
+      <c r="AN18">
+        <v>0</v>
+      </c>
+      <c r="AO18">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:41">
+      <c r="A19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" t="s">
         <v>76</v>
       </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>1</v>
-      </c>
-      <c r="G16">
-        <v>2</v>
-      </c>
-      <c r="H16" t="b">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>1</v>
-      </c>
-      <c r="J16">
-        <v>2</v>
-      </c>
-      <c r="K16" t="b">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16">
-        <v>2</v>
-      </c>
-      <c r="N16" t="b">
-        <v>0</v>
-      </c>
-      <c r="O16">
-        <v>1</v>
-      </c>
-      <c r="P16">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="b">
-        <v>1</v>
-      </c>
-      <c r="R16">
-        <v>0</v>
-      </c>
-      <c r="S16">
-        <v>0</v>
-      </c>
-      <c r="T16" t="b">
-        <v>0</v>
-      </c>
-      <c r="U16">
-        <v>1</v>
-      </c>
-      <c r="V16">
-        <v>2</v>
-      </c>
-      <c r="W16" t="b">
-        <v>0</v>
-      </c>
-      <c r="X16">
-        <v>1</v>
-      </c>
-      <c r="Y16">
-        <v>2</v>
-      </c>
-      <c r="Z16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA16">
-        <v>1</v>
-      </c>
-      <c r="AB16">
-        <v>1</v>
-      </c>
-      <c r="AC16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD16">
-        <v>1</v>
-      </c>
-      <c r="AE16">
-        <v>1</v>
-      </c>
-      <c r="AF16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG16">
-        <v>1</v>
-      </c>
-      <c r="AH16">
-        <v>2</v>
-      </c>
-      <c r="AI16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ16">
-        <v>1</v>
-      </c>
-      <c r="AK16">
-        <v>1</v>
-      </c>
-      <c r="AL16" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM16">
-        <v>0</v>
-      </c>
-      <c r="AN16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:40">
-      <c r="A17" t="s">
-        <v>55</v>
-      </c>
-      <c r="B17" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17" t="b">
-        <v>1</v>
-      </c>
-      <c r="I17">
-        <v>0</v>
-      </c>
-      <c r="J17">
-        <v>0</v>
-      </c>
-      <c r="K17" t="b">
-        <v>1</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17" t="b">
-        <v>1</v>
-      </c>
-      <c r="O17">
-        <v>0</v>
-      </c>
-      <c r="P17">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="b">
-        <v>1</v>
-      </c>
-      <c r="R17">
-        <v>0</v>
-      </c>
-      <c r="S17">
-        <v>0</v>
-      </c>
-      <c r="T17" t="b">
-        <v>1</v>
-      </c>
-      <c r="U17">
-        <v>0</v>
-      </c>
-      <c r="V17">
-        <v>0</v>
-      </c>
-      <c r="W17" t="b">
-        <v>1</v>
-      </c>
-      <c r="X17">
-        <v>0</v>
-      </c>
-      <c r="Y17">
-        <v>0</v>
-      </c>
-      <c r="Z17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA17">
-        <v>0</v>
-      </c>
-      <c r="AB17">
-        <v>0</v>
-      </c>
-      <c r="AC17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD17">
-        <v>0</v>
-      </c>
-      <c r="AE17">
-        <v>0</v>
-      </c>
-      <c r="AF17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG17">
-        <v>0</v>
-      </c>
-      <c r="AH17">
-        <v>0</v>
-      </c>
-      <c r="AI17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ17">
-        <v>0</v>
-      </c>
-      <c r="AK17">
-        <v>0</v>
-      </c>
-      <c r="AL17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM17">
-        <v>0</v>
-      </c>
-      <c r="AN17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:40">
-      <c r="A18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" t="s">
-        <v>74</v>
-      </c>
-      <c r="C18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
-      <c r="E18" t="b">
-        <v>0</v>
-      </c>
-      <c r="F18">
-        <v>1</v>
-      </c>
-      <c r="G18">
-        <v>1</v>
-      </c>
-      <c r="H18" t="b">
-        <v>0</v>
-      </c>
-      <c r="I18">
-        <v>1</v>
-      </c>
-      <c r="J18">
-        <v>1</v>
-      </c>
-      <c r="K18" t="b">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>1</v>
-      </c>
-      <c r="M18">
-        <v>2</v>
-      </c>
-      <c r="N18" t="b">
-        <v>0</v>
-      </c>
-      <c r="O18">
-        <v>1</v>
-      </c>
-      <c r="P18">
-        <v>1</v>
-      </c>
-      <c r="Q18" t="b">
-        <v>1</v>
-      </c>
-      <c r="R18">
-        <v>0</v>
-      </c>
-      <c r="S18">
-        <v>0</v>
-      </c>
-      <c r="T18" t="b">
-        <v>0</v>
-      </c>
-      <c r="U18">
-        <v>1</v>
-      </c>
-      <c r="V18">
-        <v>2</v>
-      </c>
-      <c r="W18" t="b">
-        <v>0</v>
-      </c>
-      <c r="X18">
-        <v>1</v>
-      </c>
-      <c r="Y18">
-        <v>1</v>
-      </c>
-      <c r="Z18" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA18">
-        <v>1</v>
-      </c>
-      <c r="AB18">
-        <v>1</v>
-      </c>
-      <c r="AC18" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD18">
-        <v>1</v>
-      </c>
-      <c r="AE18">
-        <v>1</v>
-      </c>
-      <c r="AF18" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG18">
-        <v>1</v>
-      </c>
-      <c r="AH18">
-        <v>2</v>
-      </c>
-      <c r="AI18" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ18">
-        <v>1</v>
-      </c>
-      <c r="AK18">
-        <v>1</v>
-      </c>
-      <c r="AL18" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM18">
-        <v>0</v>
-      </c>
-      <c r="AN18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:40">
-      <c r="A19" t="s">
-        <v>57</v>
-      </c>
-      <c r="B19" t="s">
-        <v>75</v>
-      </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -2895,6 +2952,9 @@
       </c>
       <c r="AN19">
         <v>0</v>
+      </c>
+      <c r="AO19">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>